<commit_message>
test cases for login
</commit_message>
<xml_diff>
--- a/src/test/resources/data.xlsx
+++ b/src/test/resources/data.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PRASHANT\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Zygal Automation\zygal_admin_portal\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D50B96CE-AA7C-4AD0-BA0D-5EDC2E29086C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{7B66EC9C-0B95-47F0-B7FE-D1F208F8994A}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060"/>
   </bookViews>
   <sheets>
     <sheet name="loginData" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>UserName</t>
   </si>
@@ -37,12 +36,24 @@
   </si>
   <si>
     <t>Admin@01</t>
+  </si>
+  <si>
+    <t>shivani</t>
+  </si>
+  <si>
+    <t>****1234</t>
+  </si>
+  <si>
+    <t>testing</t>
+  </si>
+  <si>
+    <t>*1Zygal007</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -81,9 +92,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -398,15 +412,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAC1EDCD-68CB-409A-A967-73E465B74E40}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="24.33203125" customWidth="1"/>
+    <col min="2" max="2" width="24.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -414,18 +428,43 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{81BCA64A-4F00-4143-A236-94B76A069EE1}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{97D96864-9248-4B9F-AEC3-3DAD2C7F3B0E}"/>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>